<commit_message>
Graphes du cockpit : plages dynamiques au lieu de references en dur
Les blocs techniques n'ont pas un nombre de lignes fixe. Le pont en a toujours
cinq et la tension trois, mais le bloc de marge suit le noeud choisi, puisque
Q_MARGE_MARQUE_2026 bascule d'axe : cinq marques a la racine, quatre campus sur
MBway, trois sur ISCOM et Ipac, deux sur Pigier et Tunon.

Cable en dur sur AK7:AK11, le graphe tracait donc trois barres vides sur Tunon,
et aurait tronque tout noeud a plus de cinq enfants.

Les douze series passent maintenant par des noms definis en OFFSET + COUNTA,
dimensionnes sur le nombre de lignes reellement remplies. Le graphe suit le
filtre sans qu'on y retouche, dans les deux sens.

Formules du tableau intactes, controle qualite toujours en PASS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/COCKPIT_nav541_MEP.xlsx
+++ b/eduservices/COCKPIT_nav541_MEP.xlsx
@@ -8,7 +8,20 @@
   <sheets>
     <sheet name="2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="pont_AD">OFFSET('2'!$AD$7,0,0,MAX(1,COUNTA('2'!$AC$7:$AC$80)),1)</definedName>
+    <definedName name="pont_AE">OFFSET('2'!$AE$7,0,0,MAX(1,COUNTA('2'!$AC$7:$AC$80)),1)</definedName>
+    <definedName name="pont_AF">OFFSET('2'!$AF$7,0,0,MAX(1,COUNTA('2'!$AC$7:$AC$80)),1)</definedName>
+    <definedName name="pont_AG">OFFSET('2'!$AG$7,0,0,MAX(1,COUNTA('2'!$AC$7:$AC$80)),1)</definedName>
+    <definedName name="pont_cat">OFFSET('2'!$AC$7,0,0,MAX(1,COUNTA('2'!$AC$7:$AC$80)),1)</definedName>
+    <definedName name="marge_AN">OFFSET('2'!$AN$7,0,0,MAX(1,COUNTA('2'!$AK$7:$AK$80)),1)</definedName>
+    <definedName name="marge_AQ">OFFSET('2'!$AQ$7,0,0,MAX(1,COUNTA('2'!$AK$7:$AK$80)),1)</definedName>
+    <definedName name="marge_AT">OFFSET('2'!$AT$7,0,0,MAX(1,COUNTA('2'!$AK$7:$AK$80)),1)</definedName>
+    <definedName name="marge_cat">OFFSET('2'!$AK$7,0,0,MAX(1,COUNTA('2'!$AK$7:$AK$80)),1)</definedName>
+    <definedName name="tension_BC">OFFSET('2'!$BC$7,0,0,MAX(1,COUNTA('2'!$AZ$7:$AZ$80)),1)</definedName>
+    <definedName name="tension_BD">OFFSET('2'!$BD$7,0,0,MAX(1,COUNTA('2'!$AZ$7:$AZ$80)),1)</definedName>
+    <definedName name="tension_cat">OFFSET('2'!$AZ$7,0,0,MAX(1,COUNTA('2'!$AZ$7:$AZ$80)),1)</definedName>
+  </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -1575,12 +1588,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AC$7:$AC$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AD$7:$AD$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_AD</f>
             </numRef>
           </val>
         </ser>
@@ -1598,12 +1611,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AC$7:$AC$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AE$7:$AE$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_AE</f>
             </numRef>
           </val>
         </ser>
@@ -1621,12 +1634,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AC$7:$AC$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AF$7:$AF$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_AF</f>
             </numRef>
           </val>
         </ser>
@@ -1644,12 +1657,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AC$7:$AC$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AG$7:$AG$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!pont_AG</f>
             </numRef>
           </val>
         </ser>
@@ -1717,12 +1730,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AK$7:$AK$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AN$7:$AN$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_AN</f>
             </numRef>
           </val>
         </ser>
@@ -1743,12 +1756,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AK$7:$AK$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AQ$7:$AQ$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_AQ</f>
             </numRef>
           </val>
         </ser>
@@ -1769,12 +1782,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'2'!$AK$7:$AK$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$AT$7:$AT$11</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!marge_AT</f>
             </numRef>
           </val>
         </ser>
@@ -1855,12 +1868,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'2'!$AZ$7:$AZ$9</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!tension_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$BC$7:$BC$9</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!tension_BC</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1896,12 +1909,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'2'!$AZ$7:$AZ$9</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!tension_cat</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'2'!$BD$7:$BD$9</f>
+              <f>'COCKPIT_nav541_MEP.xlsx'!tension_BD</f>
             </numRef>
           </val>
           <smooth val="0"/>

</xml_diff>